<commit_message>
Add quali fuel analysis, BR2 protocol support, coasting/fuel-save updates, and helper validation scripts
</commit_message>
<xml_diff>
--- a/dataAcquisition/Motec_MP/alias/eventAlias2025.xlsx
+++ b/dataAcquisition/Motec_MP/alias/eventAlias2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SimEnv\dataAcquisition\Motec_MP\alias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE66FFB-453D-4241-A139-4E446FF7DE9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDA3484-036D-4BC1-9B72-2F495B0FE724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38820" yWindow="2055" windowWidth="18180" windowHeight="13740" activeTab="2" xr2:uid="{968229EC-9479-47A1-8BEC-6418C2655BFD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{968229EC-9479-47A1-8BEC-6418C2655BFD}"/>
   </bookViews>
   <sheets>
     <sheet name="EVENT" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2688" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2688" uniqueCount="380">
   <si>
     <t>V8SC_Name</t>
   </si>
@@ -1163,6 +1163,21 @@
   </si>
   <si>
     <t>TTSO Race 22</t>
+  </si>
+  <si>
+    <t>Qualifying Race 11 Part 1</t>
+  </si>
+  <si>
+    <t>Qualifying Race 12  Part 1</t>
+  </si>
+  <si>
+    <t>Qualifying Race 12 Part 1</t>
+  </si>
+  <si>
+    <t>Qualifying Race 13 Part 1</t>
+  </si>
+  <si>
+    <t>Qualifying Race 13 Part 2</t>
   </si>
 </sst>
 </file>
@@ -2248,6 +2263,7 @@
     <col min="6" max="6" width="27.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
@@ -3564,7 +3580,7 @@
         <v>21</v>
       </c>
       <c r="E21" t="s">
-        <v>21</v>
+        <v>375</v>
       </c>
       <c r="F21" t="s">
         <v>330</v>
@@ -3629,7 +3645,7 @@
         <v>21</v>
       </c>
       <c r="E22" t="s">
-        <v>21</v>
+        <v>376</v>
       </c>
       <c r="F22" t="s">
         <v>334</v>
@@ -3647,7 +3663,7 @@
         <v>341</v>
       </c>
       <c r="K22" t="s">
-        <v>21</v>
+        <v>377</v>
       </c>
       <c r="L22" t="s">
         <v>21</v>
@@ -3694,10 +3710,10 @@
         <v>21</v>
       </c>
       <c r="E23" t="s">
-        <v>21</v>
+        <v>378</v>
       </c>
       <c r="F23" t="s">
-        <v>21</v>
+        <v>379</v>
       </c>
       <c r="G23" t="s">
         <v>21</v>

</xml_diff>